<commit_message>
First content now added
</commit_message>
<xml_diff>
--- a/classwork.xlsx
+++ b/classwork.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sir easynett\Desktop\IOTB tech\IOTB Tech Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F82840-36C6-439C-93F2-FE9997A43570}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943949A5-6A28-4646-8873-EABFC5B8123A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4470" xr2:uid="{B40EE282-128C-4E68-98A0-E13DEB69C55F}"/>
   </bookViews>
@@ -24,9 +24,17 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="1">
+  <si>
+    <t>EASYNETT COMPUTERS LIMITED</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -34,13 +42,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="0"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,8 +76,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,9 +398,38 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>